<commit_message>
Update test cases numeration
</commit_message>
<xml_diff>
--- a/test_cases.xlsx
+++ b/test_cases.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="25207"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CD4569E3-AEAC-44FB-B439-BAB819964D72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7E0A8CF1-EDFB-40C2-BFEA-EED07811A194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -92,7 +92,7 @@
     <t>Ответ: статус код HTTP - 200, в Content есть медведь с bear_id, полученный в Content в шаге 6.</t>
   </si>
   <si>
-    <t>3. Получить запись о медведе</t>
+    <t>2. Получить запись о медведе</t>
   </si>
   <si>
     <t>Предусловие: существует медведь с bear_id = ID</t>
@@ -104,7 +104,7 @@
     <t>Ответ: статус код HTTP - 200, в Content - json с bear_id = ID.</t>
   </si>
   <si>
-    <t>4. Обновить запись о медведе</t>
+    <t>3. Обновить запись о медведе</t>
   </si>
   <si>
     <t>1. Отправить PUT-запрос на эндпоинт /bear/ID</t>
@@ -158,7 +158,7 @@
     <t>Ответ: статус код HTTP - 200, в Content - json, отправленный на шаге 7 и bear_id = ID.</t>
   </si>
   <si>
-    <t>5. Удалить записи о всех медведях</t>
+    <t>4. Удалить записи о всех медведях</t>
   </si>
   <si>
     <t>Предусловие: существует хотя бы 1 медведь</t>
@@ -173,7 +173,7 @@
     <t>Ответ: статус код HTTP - 200, в Content пустой список в формате JSON.</t>
   </si>
   <si>
-    <t>6. Удалить запись о медведе</t>
+    <t>5. Удалить запись о медведе</t>
   </si>
   <si>
     <t>1. Отправить DELETE-запрос на эндпоинт /bear/ID</t>
@@ -182,7 +182,7 @@
     <t>Ответ: статус код HTTP - 200, в Content нет медведя с bear_id, равным ID</t>
   </si>
   <si>
-    <t>7. Получить несуществующую запись о медведе</t>
+    <t>6. Получить несуществующую запись о медведе</t>
   </si>
   <si>
     <t xml:space="preserve">Предусловие: медведя с bear_id = ID не существует </t>
@@ -191,7 +191,7 @@
     <t>Ответ: статус код HTTP - 200, в Content - сообщение, что записи нет</t>
   </si>
   <si>
-    <t>8. Получить пустой список медведей</t>
+    <t>7. Получить пустой список медведей</t>
   </si>
   <si>
     <t>Предусловие: записей о медведях нет</t>
@@ -200,19 +200,19 @@
     <t>1. Отправить GET-запрос на эндпоинт /bear</t>
   </si>
   <si>
-    <t>9. Обновить запись несуществующего медведя</t>
+    <t>8. Обновить запись несуществующего медведя</t>
   </si>
   <si>
     <t>Ответ: статус код HTTP - 404</t>
   </si>
   <si>
-    <t>10. Удалить запись несуществующего медведя</t>
-  </si>
-  <si>
-    <t>11. Удалить несуществующие записи о всех медведях</t>
-  </si>
-  <si>
-    <t>12. Создать медведя с частично заполненными обязательными полями</t>
+    <t>9. Удалить запись несуществующего медведя</t>
+  </si>
+  <si>
+    <t>10. Удалить несуществующие записи о всех медведях</t>
+  </si>
+  <si>
+    <t>11. Создать медведя с частично заполненными обязательными полями</t>
   </si>
   <si>
     <t>Ответ: статус код HTTP - 200, в Content - сообщение об ошибке, медведь не должен быть создан</t>
@@ -221,7 +221,7 @@
     <t>payload {"bear_name":"mikhail"}</t>
   </si>
   <si>
-    <t>13. Создать медведя с частично неверными полями</t>
+    <t>12. Создать медведя с частично неверными полями</t>
   </si>
   <si>
     <t>payload {"bear_type":"GIANT","bear_name":"Test bear name","bear_age":15.1}</t>
@@ -242,7 +242,7 @@
     <t>payload {"bear_type":"BROWN","bear_name":"Test bear name","bear_age":-10}</t>
   </si>
   <si>
-    <t>14. Создать медведя с лишними полями</t>
+    <t>13. Создать медведя с лишними полями</t>
   </si>
   <si>
     <t>Ответ: статус код HTTP - 201, в Content - число, равное ID созданного медведя, медведь должен быть создан без лишних полей</t>
@@ -251,46 +251,46 @@
     <t>payload {"Qwe": "asd", "bear_type":"BLACK","bear_name":"mikhail","bear_age":17.5}</t>
   </si>
   <si>
-    <t>15. Обновить запись медведя частично заполненными обязательными полями</t>
+    <t>14. Обновить запись медведя частично заполненными обязательными полями</t>
   </si>
   <si>
     <t>Ответ: статус код HTTP - 200, в Content - сообщение об ошибке, запись о медведе не должна измениться</t>
   </si>
   <si>
-    <t>16. Обновить запись медведя частично неверными полями</t>
+    <t>15. Обновить запись медведя частично неверными полями</t>
   </si>
   <si>
     <t>2. Отправить PUT-запрос на эндпоинт /bear</t>
   </si>
   <si>
-    <t>17. Обновить запись медведя лишними полями</t>
+    <t>16. Обновить запись медведя лишними полями</t>
   </si>
   <si>
     <t>Ответ: статус код HTTP - 200, в Content - сообщение-подтверждение, запись о медведе должна быть обновлена</t>
   </si>
   <si>
-    <t>18. Создать медведя с пустым payload</t>
-  </si>
-  <si>
-    <t>19. Создать несколько медведей за один запрос</t>
+    <t>17. Создать медведя с пустым payload</t>
+  </si>
+  <si>
+    <t>18. Создать несколько медведей за один запрос</t>
   </si>
   <si>
     <t>payload [{"bear_type":"BLACK","bear_name":"bear_1","bear_age":10}, {"bear_type":"BROWN","bear_name":"bear_2","bear_age":11}]</t>
   </si>
   <si>
-    <t>20. Создать медведя с payload в формате XML</t>
+    <t>19. Создать медведя с payload в формате XML</t>
   </si>
   <si>
     <t>payload &lt;bear&gt;&lt;bear_type&gt;BLACK&lt;/bear_type&gt;&lt;bear_name&gt;Test Name&lt;/bear_name&gt;&lt;bear_age&gt;10&lt;/bear_age&gt;&lt;/bear&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">21. Создать медведя с неправильными заголовками </t>
+    <t xml:space="preserve">20. Создать медведя с неправильными заголовками </t>
   </si>
   <si>
     <t>Content-Type: application/xml</t>
   </si>
   <si>
-    <t>22. Создать медведя с длинным именем</t>
+    <t>21. Создать медведя с длинным именем</t>
   </si>
   <si>
     <t>Ответ: статус код HTTP - 200, в Content - id созданного медведя, медведь должен быть создан с переданными данными</t>
@@ -302,16 +302,16 @@
     <t>payload {"bear_type":"BLACK","bear_name":"Long name","bear_age":17.5}</t>
   </si>
   <si>
-    <t>23. Обновить запись о медведе пустым payload</t>
-  </si>
-  <si>
-    <t>24. Обновить запись медведя списком из нескольких медведей</t>
-  </si>
-  <si>
-    <t>25. Обновить запись медведя с payload в формате XML</t>
-  </si>
-  <si>
-    <t xml:space="preserve">26. Обновить запись медведя с неправильными заголовками </t>
+    <t>22. Обновить запись о медведе пустым payload</t>
+  </si>
+  <si>
+    <t>23. Обновить запись медведя списком из нескольких медведей</t>
+  </si>
+  <si>
+    <t>24. Обновить запись медведя с payload в формате XML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">25. Обновить запись медведя с неправильными заголовками </t>
   </si>
 </sst>
 </file>

</xml_diff>